<commit_message>
Add two material May-June Meta receipts to AAA ledger and report
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DVpXqei8SkhtudMXpKxe2v
</commit_message>
<xml_diff>
--- a/invoices/exports/expenses-aaa-2026-05-06.xlsx
+++ b/invoices/exports/expenses-aaa-2026-05-06.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -572,36 +572,36 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AdEspresso</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-2108</t>
+          <t>27080113735008819-27045888015098052</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>ILS</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>2.922</v>
+        <v>3093</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>143.18</v>
+        <v>3093</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>מנוי Starter 17/5-16/6</t>
+          <t>פרסום מטא</t>
         </is>
       </c>
     </row>
@@ -613,48 +613,48 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>נת"מ ניהול צרפתי ספייס</t>
+          <t>AdEspresso</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6/2983</t>
+          <t>2026-2108</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ILS</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2929</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>1</v>
+        <v>49</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>2.922</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>2929</v>
+        <v>143.18</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>דמי אחזקה 05/26 - יגאל אלון 53 ת"א</t>
+          <t>מנוי Starter 17/5-16/6</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>נת"מ ניהול צרפתי ספייס</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>27037367769283413-27198049099881946</t>
+          <t>6/2983</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -663,24 +663,24 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2629</v>
+        <v>2929</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2629</v>
+        <v>2929</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>פרסום 14-21.5</t>
+          <t>דמי אחזקה 05/26 - יגאל אלון 53 ת"א</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>27291002590586600-27228095853543939</t>
+          <t>27037367769283413-27198049099881946</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -699,17 +699,17 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2633</v>
+        <v>2629</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>2633</v>
+        <v>2629</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>פרסום עד 27.5</t>
+          <t>פרסום 14-21.5</t>
         </is>
       </c>
     </row>
@@ -721,12 +721,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>איילה קאופמן (ayaladigital)</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>20023</t>
+          <t>27291002590586600-27228095853543939</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -735,34 +735,34 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>3304</v>
+        <v>2633</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>3304</v>
+        <v>2633</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>קבלה - שיווק דיגיטלי פייסבוק מאי (חשבונית 10026)</t>
+          <t>פרסום עד 27.5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>א.מ.י טכנולוגיות רפואיות</t>
+          <t>איילה קאופמן (ayaladigital)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SI26019672</t>
+          <t>20023</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -771,34 +771,34 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>614</v>
+        <v>3304</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>614</v>
+        <v>3304</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>חשבונית מרכזת - מופיע גם בדוח המייל האישי</t>
+          <t>קבלה - שיווק דיגיטלי פייסבוק מאי (חשבונית 10026)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>א.מ.י טכנולוגיות רפואיות</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SI26019671</t>
+          <t>27375940462092812-27233538499666336</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -807,17 +807,17 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>5039</v>
+        <v>2633</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>5039</v>
+        <v>2633</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>חשבונית מרכזת - מופיע גם בדוח המייל האישי</t>
+          <t>פרסום מטא</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SI26019663</t>
+          <t>SI26019672</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -843,13 +843,13 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>10148</v>
+        <v>614</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>10148</v>
+        <v>614</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SI26019650</t>
+          <t>SI26019671</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -879,13 +879,13 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>472</v>
+        <v>5039</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>472</v>
+        <v>5039</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SI26019641</t>
+          <t>SI26019663</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -915,13 +915,13 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>2867</v>
+        <v>10148</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>2867</v>
+        <v>10148</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -932,17 +932,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>א.מ.י טכנולוגיות רפואיות</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>27292304737123046-27306268615726657</t>
+          <t>SI26019650</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -951,24 +951,24 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>2095.01</v>
+        <v>472</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>2095.01</v>
+        <v>472</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>פרסום 31.5-6.6</t>
+          <t>חשבונית מרכזת - מופיע גם בדוח המייל האישי</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SI26020048</t>
+          <t>SI26019641</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -987,24 +987,24 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>7080</v>
+        <v>2867</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>7080</v>
+        <v>2867</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>מזרקי Sculptra - מופיע גם בדוח המייל האישי</t>
+          <t>חשבונית מרכזת - מופיע גם בדוח המייל האישי</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>27475702388783283-27442231395463710</t>
+          <t>27292304737123046-27306268615726657</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1023,34 +1023,34 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2677</v>
+        <v>2095.01</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>2677</v>
+        <v>2095.01</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>פרסום 7-13.6</t>
+          <t>פרסום 31.5-6.6</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>נת"מ ניהול צרפתי ספייס</t>
+          <t>א.מ.י טכנולוגיות רפואיות</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>6/3065</t>
+          <t>SI26020048</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1059,24 +1059,24 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>2929</v>
+        <v>7080</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>2929</v>
+        <v>7080</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>דמי אחזקה 06/26</t>
+          <t>מזרקי Sculptra - מופיע גם בדוח המייל האישי</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>27425698177117033-27505252845828237</t>
+          <t>27475702388783283-27442231395463710</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1095,34 +1095,34 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>2.18</v>
+        <v>2677</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>2.18</v>
+        <v>2677</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>קרדיט פרסום 15.6</t>
+          <t>פרסום 7-13.6</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>נת"מ ניהול צרפתי ספייס</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27459771810376342-27507624268924422</t>
+          <t>6/3065</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1131,34 +1131,34 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2677</v>
+        <v>2929</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2677</v>
+        <v>2929</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>פרסום מטא</t>
+          <t>דמי אחזקה 06/26</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>איילה קאופמן (ayaladigital)</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>30191</t>
+          <t>27425698177117033-27505252845828237</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1167,34 +1167,34 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>3304</v>
+        <v>2.18</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>3304</v>
+        <v>2.18</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה - שיווק דיגיטלי פייסבוק יוני</t>
+          <t>קרדיט פרסום 15.6</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>Meta Ads (בית ספר לרפואה אסתטית)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27520586224294900-27667611399592382</t>
+          <t>27518269867859868-27393420967011423</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1203,78 +1203,186 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>2677</v>
+        <v>0.91</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>2677</v>
+        <v>0.91</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>פרסום מטא</t>
+          <t>קרדיט פרסום</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Meta Ads (601049505664355)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>27459771810376342-27507624268924422</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>2677</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>2677</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>פרסום מטא</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>איילה קאופמן (ayaladigital)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>30191</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>3304</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>3304</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>חשבונית מס קבלה - שיווק דיגיטלי פייסבוק יוני</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Meta Ads (601049505664355)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>27520586224294900-27667611399592382</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>2677</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>2677</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>פרסום מטא</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>27663629833323869-27582126164807572</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>ILS</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
         <v>2701</v>
       </c>
-      <c r="F22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="2" t="n">
+      <c r="F25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2" t="n">
         <v>2701</v>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>פרסום מטא</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="5" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>סה"כ בש"ח</t>
         </is>
       </c>
-      <c r="G24" s="6" t="n">
-        <v>57301.55</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="7" t="inlineStr">
+      <c r="G27" s="6" t="n">
+        <v>63028.46</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>מזה חשבוניות AMI שמופיעות גם בדוח מהמייל האישי (לספור פעם אחת)</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>26220</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>המרות מט"ח לפי שער יציג יומי ליום המסמך. קבלות Meta של חשבון גלונס אסתטיקה מופיעות בדוח האישי בלבד.</t>
         </is>

</xml_diff>

<commit_message>
Add May 6 Meta receipt to AAA ledger and report
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DVpXqei8SkhtudMXpKxe2v
</commit_message>
<xml_diff>
--- a/invoices/exports/expenses-aaa-2026-05-06.xlsx
+++ b/invoices/exports/expenses-aaa-2026-05-06.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>26824808960539292-26884582841228572</t>
+          <t>27014420118244850-26951644557855738</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -519,34 +519,34 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>246.03</v>
+        <v>3093</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>246.03</v>
+        <v>3093</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>פרסום 5-6.5 קמפיין איילה לידים</t>
+          <t>פרסום מטא</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Meta Ads (382848224834261)</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>26962869060069675-27054348037588449</t>
+          <t>26824808960539292-26884582841228572</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -555,17 +555,17 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>135.15</v>
+        <v>246.03</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>135.15</v>
+        <v>246.03</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>פרסום - קמפיין STRA הסמכה לבוגרי רפואה</t>
+          <t>פרסום 5-6.5 קמפיין איילה לידים</t>
         </is>
       </c>
     </row>
@@ -577,12 +577,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>Meta Ads (382848224834261)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27080113735008819-27045888015098052</t>
+          <t>26962869060069675-27054348037588449</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -591,53 +591,53 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3093</v>
+        <v>135.15</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>3093</v>
+        <v>135.15</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>פרסום מטא</t>
+          <t>פרסום - קמפיין STRA הסמכה לבוגרי רפואה</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AdEspresso</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-2108</t>
+          <t>27080113735008819-27045888015098052</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>ILS</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>2.922</v>
+        <v>3093</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>143.18</v>
+        <v>3093</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>מנוי Starter 17/5-16/6</t>
+          <t>פרסום מטא</t>
         </is>
       </c>
     </row>
@@ -649,48 +649,48 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>נת"מ ניהול צרפתי ספייס</t>
+          <t>AdEspresso</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>6/2983</t>
+          <t>2026-2108</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ILS</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2929</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>1</v>
+        <v>49</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>2.922</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2929</v>
+        <v>143.18</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>דמי אחזקה 05/26 - יגאל אלון 53 ת"א</t>
+          <t>מנוי Starter 17/5-16/6</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>נת"מ ניהול צרפתי ספייס</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>27037367769283413-27198049099881946</t>
+          <t>6/2983</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -699,24 +699,24 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2629</v>
+        <v>2929</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>2629</v>
+        <v>2929</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>פרסום 14-21.5</t>
+          <t>דמי אחזקה 05/26 - יגאל אלון 53 ת"א</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>27291002590586600-27228095853543939</t>
+          <t>27037367769283413-27198049099881946</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -735,17 +735,17 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>2633</v>
+        <v>2629</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>2633</v>
+        <v>2629</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>פרסום עד 27.5</t>
+          <t>פרסום 14-21.5</t>
         </is>
       </c>
     </row>
@@ -757,12 +757,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>איילה קאופמן (ayaladigital)</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>20023</t>
+          <t>27291002590586600-27228095853543939</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -771,34 +771,34 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3304</v>
+        <v>2633</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>3304</v>
+        <v>2633</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>קבלה - שיווק דיגיטלי פייסבוק מאי (חשבונית 10026)</t>
+          <t>פרסום עד 27.5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>איילה קאופמן (ayaladigital)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>27375940462092812-27233538499666336</t>
+          <t>20023</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -807,34 +807,34 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2633</v>
+        <v>3304</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>2633</v>
+        <v>3304</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>פרסום מטא</t>
+          <t>קבלה - שיווק דיגיטלי פייסבוק מאי (חשבונית 10026)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>א.מ.י טכנולוגיות רפואיות</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SI26019672</t>
+          <t>27375940462092812-27233538499666336</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -843,17 +843,17 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>614</v>
+        <v>2633</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>614</v>
+        <v>2633</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>חשבונית מרכזת - מופיע גם בדוח המייל האישי</t>
+          <t>פרסום מטא</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SI26019671</t>
+          <t>SI26019672</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -879,13 +879,13 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5039</v>
+        <v>614</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>5039</v>
+        <v>614</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SI26019663</t>
+          <t>SI26019671</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -915,13 +915,13 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>10148</v>
+        <v>5039</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>10148</v>
+        <v>5039</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -942,7 +942,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SI26019650</t>
+          <t>SI26019663</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -951,13 +951,13 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>472</v>
+        <v>10148</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>472</v>
+        <v>10148</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SI26019641</t>
+          <t>SI26019650</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -987,13 +987,13 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2867</v>
+        <v>472</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>2867</v>
+        <v>472</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1004,17 +1004,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>א.מ.י טכנולוגיות רפואיות</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>27292304737123046-27306268615726657</t>
+          <t>SI26019641</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1023,34 +1023,34 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2095.01</v>
+        <v>2867</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>2095.01</v>
+        <v>2867</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>פרסום 31.5-6.6</t>
+          <t>חשבונית מרכזת - מופיע גם בדוח המייל האישי</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>א.מ.י טכנולוגיות רפואיות</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SI26020048</t>
+          <t>27292304737123046-27306268615726657</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1059,34 +1059,34 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>7080</v>
+        <v>2095.01</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>7080</v>
+        <v>2095.01</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>מזרקי Sculptra - מופיע גם בדוח המייל האישי</t>
+          <t>פרסום 31.5-6.6</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>א.מ.י טכנולוגיות רפואיות</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>27475702388783283-27442231395463710</t>
+          <t>SI26020048</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1095,34 +1095,34 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>2677</v>
+        <v>7080</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>2677</v>
+        <v>7080</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>פרסום 7-13.6</t>
+          <t>מזרקי Sculptra - מופיע גם בדוח המייל האישי</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>נת"מ ניהול צרפתי ספייס</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>6/3065</t>
+          <t>27475702388783283-27442231395463710</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1131,34 +1131,34 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2929</v>
+        <v>2677</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2929</v>
+        <v>2677</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>דמי אחזקה 06/26</t>
+          <t>פרסום 7-13.6</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>נת"מ ניהול צרפתי ספייס</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27425698177117033-27505252845828237</t>
+          <t>6/3065</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1167,34 +1167,34 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2.18</v>
+        <v>2929</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>2.18</v>
+        <v>2929</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>קרדיט פרסום 15.6</t>
+          <t>דמי אחזקה 06/26</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Meta Ads (בית ספר לרפואה אסתטית)</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27518269867859868-27393420967011423</t>
+          <t>27425698177117033-27505252845828237</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1203,34 +1203,34 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.91</v>
+        <v>2.18</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.91</v>
+        <v>2.18</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>קרדיט פרסום</t>
+          <t>קרדיט פרסום 15.6</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>Meta Ads (בית ספר לרפואה אסתטית)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27459771810376342-27507624268924422</t>
+          <t>27518269867859868-27393420967011423</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1239,34 +1239,34 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2677</v>
+        <v>0.91</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>2677</v>
+        <v>0.91</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>פרסום מטא</t>
+          <t>קרדיט פרסום</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>איילה קאופמן (ayaladigital)</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>30191</t>
+          <t>27459771810376342-27507624268924422</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1275,34 +1275,34 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>3304</v>
+        <v>2677</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>3304</v>
+        <v>2677</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה - שיווק דיגיטלי פייסבוק יוני</t>
+          <t>פרסום מטא</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>איילה קאופמן (ayaladigital)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>27520586224294900-27667611399592382</t>
+          <t>30191</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1311,78 +1311,114 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>2677</v>
+        <v>3304</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>2677</v>
+        <v>3304</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>פרסום מטא</t>
+          <t>חשבונית מס קבלה - שיווק דיגיטלי פייסבוק יוני</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Meta Ads (601049505664355)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>27520586224294900-27667611399592382</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>2677</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>2677</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>פרסום מטא</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>27663629833323869-27582126164807572</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>ILS</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
         <v>2701</v>
       </c>
-      <c r="F25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="2" t="n">
+      <c r="F26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2" t="n">
         <v>2701</v>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>פרסום מטא</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="5" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>סה"כ בש"ח</t>
         </is>
       </c>
-      <c r="G27" s="6" t="n">
-        <v>63028.46</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="7" t="inlineStr">
+      <c r="G28" s="6" t="n">
+        <v>66121.46000000001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>מזה חשבוניות AMI שמופיעות גם בדוח מהמייל האישי (לספור פעם אחת)</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>26220</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>המרות מט"ח לפי שער יציג יומי ליום המסמך. קבלות Meta של חשבון גלונס אסתטיקה מופיעות בדוח האישי בלבד.</t>
         </is>

</xml_diff>

<commit_message>
Add June 8 and April Meta receipts to AAA ledger
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DVpXqei8SkhtudMXpKxe2v
</commit_message>
<xml_diff>
--- a/invoices/exports/expenses-aaa-2026-05-06.xlsx
+++ b/invoices/exports/expenses-aaa-2026-05-06.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1081,12 +1081,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>א.מ.י טכנולוגיות רפואיות</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SI26020048</t>
+          <t>27440847285602125-27264069279946589</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1095,34 +1095,34 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>7080</v>
+        <v>798.5</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>7080</v>
+        <v>798.5</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>מזרקי Sculptra - מופיע גם בדוח המייל האישי</t>
+          <t>פרסום מטא</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>א.מ.י טכנולוגיות רפואיות</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27475702388783283-27442231395463710</t>
+          <t>SI26020048</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1131,34 +1131,34 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2677</v>
+        <v>7080</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2677</v>
+        <v>7080</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>פרסום 7-13.6</t>
+          <t>מזרקי Sculptra - מופיע גם בדוח המייל האישי</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>נת"מ ניהול צרפתי ספייס</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>6/3065</t>
+          <t>27475702388783283-27442231395463710</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1167,34 +1167,34 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2929</v>
+        <v>2677</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>2929</v>
+        <v>2677</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>דמי אחזקה 06/26</t>
+          <t>פרסום 7-13.6</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>נת"מ ניהול צרפתי ספייס</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27425698177117033-27505252845828237</t>
+          <t>6/3065</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1203,34 +1203,34 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>2.18</v>
+        <v>2929</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>2.18</v>
+        <v>2929</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>קרדיט פרסום 15.6</t>
+          <t>דמי אחזקה 06/26</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Meta Ads (בית ספר לרפואה אסתטית)</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27518269867859868-27393420967011423</t>
+          <t>27425698177117033-27505252845828237</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1239,34 +1239,34 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.91</v>
+        <v>2.18</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.91</v>
+        <v>2.18</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>קרדיט פרסום</t>
+          <t>קרדיט פרסום 15.6</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>Meta Ads (בית ספר לרפואה אסתטית)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>27459771810376342-27507624268924422</t>
+          <t>27518269867859868-27393420967011423</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1275,34 +1275,34 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>2677</v>
+        <v>0.91</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>2677</v>
+        <v>0.91</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>פרסום מטא</t>
+          <t>קרדיט פרסום</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>איילה קאופמן (ayaladigital)</t>
+          <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>30191</t>
+          <t>27459771810376342-27507624268924422</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1311,34 +1311,34 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>3304</v>
+        <v>2677</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>3304</v>
+        <v>2677</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>חשבונית מס קבלה - שיווק דיגיטלי פייסבוק יוני</t>
+          <t>פרסום מטא</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Meta Ads (601049505664355)</t>
+          <t>איילה קאופמן (ayaladigital)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>27520586224294900-27667611399592382</t>
+          <t>30191</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1347,78 +1347,114 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>2677</v>
+        <v>3304</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>2677</v>
+        <v>3304</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>פרסום מטא</t>
+          <t>חשבונית מס קבלה - שיווק דיגיטלי פייסבוק יוני</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Meta Ads (601049505664355)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>27520586224294900-27667611399592382</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>2677</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>2677</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>פרסום מטא</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Meta Ads (601049505664355)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>27663629833323869-27582126164807572</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>ILS</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n">
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
         <v>2701</v>
       </c>
-      <c r="F26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="2" t="n">
+      <c r="F27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="2" t="n">
         <v>2701</v>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>פרסום מטא</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="5" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>סה"כ בש"ח</t>
         </is>
       </c>
-      <c r="G28" s="6" t="n">
-        <v>66121.46000000001</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="7" t="inlineStr">
+      <c r="G29" s="6" t="n">
+        <v>66919.96000000001</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>מזה חשבוניות AMI שמופיעות גם בדוח מהמייל האישי (לספור פעם אחת)</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>26220</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>המרות מט"ח לפי שער יציג יומי ליום המסמך. קבלות Meta של חשבון גלונס אסתטיקה מופיעות בדוח האישי בלבד.</t>
         </is>

</xml_diff>